<commit_message>
paper run 2026-09-18 17:54
</commit_message>
<xml_diff>
--- a/reports/2026-09-18.xlsx
+++ b/reports/2026-09-18.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,6 +558,135 @@
       </c>
       <c r="K3" t="n">
         <v>2.4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-18T14:41:49.134975+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F4" t="n">
+        <v>56.79</v>
+      </c>
+      <c r="G4" t="n">
+        <v>105.17</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.784</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.00159</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>48.38</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-18T15:38:49.009489+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F5" t="n">
+        <v>12.96</v>
+      </c>
+      <c r="G5" t="n">
+        <v>24</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-0.00106</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>11.04</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-18T16:41:16.001610+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F6" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="G6" t="n">
+        <v>35</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.771</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-0.00152</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>15.4</v>
       </c>
     </row>
   </sheetData>
@@ -571,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -593,7 +722,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -603,7 +732,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -623,7 +752,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="6">
@@ -633,7 +762,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-1.25</v>
+        <v>73.56999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -643,7 +772,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2.4</v>
+        <v>77.22</v>
       </c>
     </row>
     <row r="8">
@@ -663,7 +792,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.66</v>
+        <v>21.16</v>
       </c>
     </row>
     <row r="10">
@@ -673,7 +802,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1135.86</v>
+        <v>1210.68</v>
       </c>
     </row>
     <row r="12">
@@ -724,16 +853,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D15" t="n">
-        <v>32.85</v>
+        <v>266.94</v>
       </c>
       <c r="E15" t="n">
-        <v>-1.25</v>
+        <v>62.53</v>
       </c>
     </row>
     <row r="16">
@@ -743,16 +872,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D16" t="n">
-        <v>33.05</v>
+        <v>110.57</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>11.04</v>
       </c>
     </row>
     <row r="17">
@@ -765,256 +894,272 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>52.32</v>
+        <v>97.84</v>
       </c>
       <c r="E18" t="n">
-        <v>2.4</v>
+        <v>59.42</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>-65.75</v>
+        <v>96.95</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>79.33</v>
+        <v>-140.17</v>
       </c>
       <c r="E20" t="n">
-        <v>-3.65</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>10</v>
+      </c>
+      <c r="C21" t="n">
+        <v>9</v>
+      </c>
+      <c r="D21" t="n">
+        <v>322.89</v>
+      </c>
+      <c r="E21" t="n">
+        <v>11.75</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>6</v>
-      </c>
-      <c r="C22" t="n">
-        <v>4</v>
-      </c>
-      <c r="D22" t="n">
-        <v>83.2</v>
-      </c>
-      <c r="E22" t="n">
-        <v>-1.25</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D23" t="n">
-        <v>-52.57</v>
+        <v>181.04</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>58.17</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D24" t="n">
-        <v>35.27</v>
+        <v>53.48</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>4</v>
+      </c>
+      <c r="C25" t="n">
+        <v>4</v>
+      </c>
+      <c r="D25" t="n">
+        <v>142.99</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>6</v>
-      </c>
-      <c r="C26" t="n">
-        <v>4</v>
-      </c>
-      <c r="D26" t="n">
-        <v>70.44</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0</v>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MAX_PER_WINDOW</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" t="n">
         <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>-4.54</v>
+        <v>44.63</v>
       </c>
       <c r="E27" t="n">
-        <v>-1.25</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>14</v>
+      </c>
+      <c r="C28" t="n">
+        <v>10</v>
+      </c>
+      <c r="D28" t="n">
+        <v>193.52</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>5</v>
+      </c>
+      <c r="C29" t="n">
+        <v>4</v>
+      </c>
+      <c r="D29" t="n">
+        <v>139.36</v>
+      </c>
+      <c r="E29" t="n">
+        <v>73.56999999999999</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>ETH</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" t="n">
-        <v>2.4</v>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>XRP</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>1</v>
-      </c>
-      <c r="C33" t="n">
-        <v>0</v>
-      </c>
-      <c r="D33" t="n">
-        <v>-3.65</v>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" t="n">
+        <v>59.42</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>2.4</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>15m</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1024,13 +1169,13 @@
         <v>1</v>
       </c>
       <c r="D36" t="n">
-        <v>-1.25</v>
+        <v>11.75</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>По часам</t>
+          <t>По окнам</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1052,23 +1197,23 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>00</t>
+          <t>15m</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D39" t="n">
-        <v>-3.65</v>
+        <v>62.53</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>5m</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1078,13 +1223,13 @@
         <v>1</v>
       </c>
       <c r="D40" t="n">
-        <v>2.4</v>
+        <v>11.04</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>По цене входа</t>
+          <t>По часам</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1106,61 +1251,71 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>00</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D43" t="n">
-        <v>-1.25</v>
+        <v>-3.65</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>2.4</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>48.38</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>1</v>
       </c>
       <c r="C46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D46" t="n">
-        <v>-3.65</v>
+        <v>11.04</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0.20%+</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1170,13 +1325,13 @@
         <v>1</v>
       </c>
       <c r="D47" t="n">
-        <v>2.4</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>По направлению</t>
+          <t>По цене входа</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1198,17 +1353,157 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>4</v>
+      </c>
+      <c r="C50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D50" t="n">
+        <v>58.17</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
+        <v>15.4</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>2</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" t="n">
+        <v>7.39</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" t="n">
+        <v>63.78</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>0.20%+</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>1</v>
+      </c>
+      <c r="C56" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B50" t="n">
-        <v>2</v>
-      </c>
-      <c r="C50" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" t="n">
-        <v>-1.25</v>
+      <c r="B59" t="n">
+        <v>4</v>
+      </c>
+      <c r="C59" t="n">
+        <v>3</v>
+      </c>
+      <c r="D59" t="n">
+        <v>25.19</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>1</v>
+      </c>
+      <c r="C60" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" t="n">
+        <v>48.38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-09-18 23:52
</commit_message>
<xml_diff>
--- a/reports/2026-09-18.xlsx
+++ b/reports/2026-09-18.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -687,6 +687,49 @@
       </c>
       <c r="K6" t="n">
         <v>15.4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-18T19:41:18.602452+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F7" t="n">
+        <v>9.18</v>
+      </c>
+      <c r="G7" t="n">
+        <v>18</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.759</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.00111</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>8.82</v>
       </c>
     </row>
   </sheetData>
@@ -700,7 +743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -722,7 +765,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -732,7 +775,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -752,7 +795,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.8</v>
+        <v>0.8333333333333334</v>
       </c>
     </row>
     <row r="6">
@@ -762,7 +805,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>73.56999999999999</v>
+        <v>82.39</v>
       </c>
     </row>
     <row r="7">
@@ -772,7 +815,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>77.22</v>
+        <v>86.04000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -792,7 +835,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>21.16</v>
+        <v>23.57</v>
       </c>
     </row>
     <row r="10">
@@ -802,7 +845,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1210.68</v>
+        <v>1219.5</v>
       </c>
     </row>
     <row r="12">
@@ -853,16 +896,16 @@
         </is>
       </c>
       <c r="B15" t="n">
+        <v>17</v>
+      </c>
+      <c r="C15" t="n">
         <v>13</v>
       </c>
-      <c r="C15" t="n">
-        <v>10</v>
-      </c>
       <c r="D15" t="n">
-        <v>266.94</v>
+        <v>374.08</v>
       </c>
       <c r="E15" t="n">
-        <v>62.53</v>
+        <v>71.34999999999999</v>
       </c>
     </row>
     <row r="16">
@@ -917,16 +960,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D19" t="n">
-        <v>96.95</v>
+        <v>155.11</v>
       </c>
       <c r="E19" t="n">
-        <v>2.4</v>
+        <v>11.22</v>
       </c>
     </row>
     <row r="20">
@@ -936,13 +979,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D20" t="n">
-        <v>-140.17</v>
+        <v>-82.01000000000001</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -955,13 +998,13 @@
         </is>
       </c>
       <c r="B21" t="n">
+        <v>12</v>
+      </c>
+      <c r="C21" t="n">
         <v>10</v>
       </c>
-      <c r="C21" t="n">
-        <v>9</v>
-      </c>
       <c r="D21" t="n">
-        <v>322.89</v>
+        <v>313.71</v>
       </c>
       <c r="E21" t="n">
         <v>11.75</v>
@@ -981,16 +1024,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C23" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D23" t="n">
-        <v>181.04</v>
+        <v>288.18</v>
       </c>
       <c r="E23" t="n">
-        <v>58.17</v>
+        <v>66.98999999999999</v>
       </c>
     </row>
     <row r="24">
@@ -1045,13 +1088,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" t="n">
-        <v>44.63</v>
+        <v>102.79</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
@@ -1064,13 +1107,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C28" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D28" t="n">
-        <v>193.52</v>
+        <v>184.34</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
@@ -1083,16 +1126,16 @@
         </is>
       </c>
       <c r="B29" t="n">
+        <v>6</v>
+      </c>
+      <c r="C29" t="n">
         <v>5</v>
       </c>
-      <c r="C29" t="n">
-        <v>4</v>
-      </c>
       <c r="D29" t="n">
-        <v>139.36</v>
+        <v>197.52</v>
       </c>
       <c r="E29" t="n">
-        <v>73.56999999999999</v>
+        <v>82.39</v>
       </c>
     </row>
     <row r="31">
@@ -1147,13 +1190,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D35" t="n">
-        <v>2.4</v>
+        <v>11.22</v>
       </c>
     </row>
     <row r="36">
@@ -1201,13 +1244,13 @@
         </is>
       </c>
       <c r="B39" t="n">
+        <v>5</v>
+      </c>
+      <c r="C39" t="n">
         <v>4</v>
       </c>
-      <c r="C39" t="n">
-        <v>3</v>
-      </c>
       <c r="D39" t="n">
-        <v>62.53</v>
+        <v>71.34999999999999</v>
       </c>
     </row>
     <row r="40">
@@ -1328,182 +1371,198 @@
         <v>15.4</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>8.82</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>4</v>
-      </c>
-      <c r="C50" t="n">
-        <v>3</v>
-      </c>
-      <c r="D50" t="n">
-        <v>58.17</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>5</v>
+      </c>
+      <c r="C51" t="n">
+        <v>4</v>
+      </c>
+      <c r="D51" t="n">
+        <v>66.98999999999999</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>0.55–0.60</t>
         </is>
       </c>
-      <c r="B51" t="n">
-        <v>1</v>
-      </c>
-      <c r="C51" t="n">
-        <v>1</v>
-      </c>
-      <c r="D51" t="n">
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
         <v>15.4</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>2</v>
-      </c>
-      <c r="C54" t="n">
-        <v>1</v>
-      </c>
-      <c r="D54" t="n">
-        <v>7.39</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>0.15–0.20%</t>
+          <t>0.10–0.12%</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C55" t="n">
         <v>2</v>
       </c>
       <c r="D55" t="n">
-        <v>63.78</v>
+        <v>16.21</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>2</v>
+      </c>
+      <c r="C56" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" t="n">
+        <v>63.78</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>0.20%+</t>
         </is>
       </c>
-      <c r="B56" t="n">
-        <v>1</v>
-      </c>
-      <c r="C56" t="n">
-        <v>1</v>
-      </c>
-      <c r="D56" t="n">
+      <c r="B57" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" t="n">
         <v>2.4</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>4</v>
-      </c>
-      <c r="C59" t="n">
-        <v>3</v>
-      </c>
-      <c r="D59" t="n">
-        <v>25.19</v>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>4</v>
+      </c>
+      <c r="C60" t="n">
+        <v>3</v>
+      </c>
+      <c r="D60" t="n">
+        <v>25.19</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B60" t="n">
-        <v>1</v>
-      </c>
-      <c r="C60" t="n">
-        <v>1</v>
-      </c>
-      <c r="D60" t="n">
-        <v>48.38</v>
+      <c r="B61" t="n">
+        <v>2</v>
+      </c>
+      <c r="C61" t="n">
+        <v>2</v>
+      </c>
+      <c r="D61" t="n">
+        <v>57.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>